<commit_message>
Day : 10 - 12 : Learn Pandas
</commit_message>
<xml_diff>
--- a/Pandas/data.xlsx
+++ b/Pandas/data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Minato\Desktop\Data Science\Pandas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6A1D9D88-51A9-4FEB-A0E9-29A0C7041D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6438B80B-A4B4-45B5-8F78-9A8C9414C196}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D3564B50-82CD-4FE0-A597-FE85AB5A9C38}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{D3564B50-82CD-4FE0-A597-FE85AB5A9C38}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="School_student" sheetId="1" r:id="rId1"/>
+    <sheet name="College_student" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>School</t>
   </si>
@@ -93,6 +94,21 @@
   </si>
   <si>
     <t>CRS</t>
+  </si>
+  <si>
+    <t>College</t>
+  </si>
+  <si>
+    <t>sem</t>
+  </si>
+  <si>
+    <t>Mahesh</t>
+  </si>
+  <si>
+    <t>Babu</t>
+  </si>
+  <si>
+    <t>PDEU</t>
   </si>
 </sst>
 </file>
@@ -569,4 +585,47 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8DEEBB1-BE1B-4658-A9A1-C9434E8F7B2D}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>